<commit_message>
Product 5.0 Home Phase 1
</commit_message>
<xml_diff>
--- a/spreadsheet/SIMS-Blog-Manager.xlsx
+++ b/spreadsheet/SIMS-Blog-Manager.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheets>
-    <sheet name="Home" sheetId="1" ns1:id="Rbf9b17eb7f704d3a"/>
-    <sheet name="今日の改善" sheetId="2" ns1:id="R360653011a78458f"/>
-    <sheet name="改善中" sheetId="3" ns1:id="R7764b58312754340"/>
-    <sheet name="ブログ診断" sheetId="4" ns1:id="R6ad346414db54781"/>
-    <sheet name="処理ログ" sheetId="5" ns1:id="Rdb636092630f4919"/>
-    <sheet name="設定" sheetId="6" ns1:id="R5fd6d2bdd543499b" state="hidden"/>
-    <sheet name="SearchConsole_Data" sheetId="7" ns1:id="R4d7533b2c69f458b" state="hidden"/>
-    <sheet name="Improvement_Queue" sheetId="8" ns1:id="R9176cfff330c4b06" state="hidden"/>
-    <sheet name="Improvement_Log" sheetId="9" ns1:id="R110f8c19d34d4160" state="hidden"/>
-  </sheets>
-</workbook>
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Home" sheetId="1" r:id="R6fc33a1f713a465a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rb8b33ffe38954ab9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善中" sheetId="3" r:id="R3f816bb506274693"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ブログ診断" sheetId="4" r:id="R9048189f3efd47c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="処理ログ" sheetId="5" r:id="R7b2b3132cb2547f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設定" sheetId="6" r:id="R6ed0b4f365394cdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SearchConsole_Data" sheetId="7" r:id="R3885d4aadad84e78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Queue" sheetId="8" r:id="R1d3c6cd1b1c44e66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Log" sheetId="9" r:id="R1189022717c94630"/>
+  </x:sheets>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -48,8 +48,46 @@
       <x:color rgb="FF17365D"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF4B5563"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F4E79"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="20"/>
+      <x:color rgb="FF111827"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF6B7280"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF111827"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF9A3412"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -71,15 +109,58 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E79"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F4F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE5E7EB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7ED"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="5">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFB7C9D6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFE5E7EB"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFE5E7EB"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE5E7EB"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="42">
+  <x:cellXfs count="88">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -173,6 +254,112 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -331,209 +518,304 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="3" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="34" t="str">
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="47" t="str">
         <x:v>SIMS-Blog-Manager Product 5.0 Official</x:v>
       </x:c>
-      <x:c r="B1" s="35"/>
-      <x:c r="C1" s="35"/>
-      <x:c r="D1" s="35"/>
-      <x:c r="E1" s="35"/>
-      <x:c r="F1" s="35"/>
-      <x:c r="G1" s="35"/>
-      <x:c r="H1" s="35"/>
+      <x:c r="B1" s="47"/>
+      <x:c r="C1" s="47"/>
+      <x:c r="D1" s="47"/>
+      <x:c r="E1" s="47"/>
+      <x:c r="F1" s="47"/>
+      <x:c r="G1" s="47"/>
+      <x:c r="H1" s="47"/>
       <x:c r="I1" s="35"/>
       <x:c r="J1" s="35"/>
       <x:c r="K1" s="35"/>
     </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="50" t="str">
+        <x:v>毎日最初に見る画面：ブログ全体・改善状況・今日やることだけを表示します。</x:v>
+      </x:c>
+      <x:c r="B2" s="50"/>
+      <x:c r="C2" s="50"/>
+      <x:c r="D2" s="50"/>
+      <x:c r="E2" s="50"/>
+      <x:c r="F2" s="50"/>
+      <x:c r="G2" s="50"/>
+      <x:c r="H2" s="50"/>
+    </x:row>
     <x:row r="3">
-      <x:c r="A3" s="13" t="str">
-        <x:v>ブログ全体の状況</x:v>
-      </x:c>
-      <x:c r="B3" s="13" t="str">
-        <x:v>件数</x:v>
-      </x:c>
-      <x:c r="C3" s="13" t="str">
-        <x:v>確認先</x:v>
-      </x:c>
-      <x:c r="E3" s="13" t="str">
+      <x:c r="A3" s="13"/>
+      <x:c r="B3" s="13"/>
+      <x:c r="C3" s="13"/>
+      <x:c r="E3" s="13"/>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="55" t="str">
+        <x:v>良好記事数</x:v>
+      </x:c>
+      <x:c r="B4" s="55"/>
+      <x:c r="C4"/>
+      <x:c r="D4" s="55" t="str">
+        <x:v>改善中記事数</x:v>
+      </x:c>
+      <x:c r="E4" s="55"/>
+      <x:c r="F4" s="20"/>
+      <x:c r="G4" s="55" t="str">
+        <x:v>改善候補数</x:v>
+      </x:c>
+      <x:c r="H4" s="55"/>
+    </x:row>
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="62" t="n">
+        <x:f>COUNTIF('ブログ診断'!$A:$A,"良好")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B5" s="62"/>
+      <x:c r="C5"/>
+      <x:c r="D5" s="62" t="n">
+        <x:f>COUNTA('改善中'!$B$2:$B$1000)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="62"/>
+      <x:c r="F5"/>
+      <x:c r="G5" s="62" t="n">
+        <x:f>COUNTIFS(Improvement_Queue!$B:$B,"&lt;&gt;",Improvement_Queue!$I:$I,"&lt;&gt;改善中",Improvement_Queue!$I:$I,"&lt;&gt;測定中",Improvement_Queue!$I:$I,"&lt;&gt;良好",Improvement_Queue!$I:$I,"&lt;&gt;改善不要")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H5" s="62"/>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="65" t="str">
+        <x:v>当面の改善不要</x:v>
+      </x:c>
+      <x:c r="B6" s="65"/>
+      <x:c r="C6"/>
+      <x:c r="D6" s="65" t="str">
+        <x:v>週1回・最大2か月測定</x:v>
+      </x:c>
+      <x:c r="E6" s="65"/>
+      <x:c r="F6"/>
+      <x:c r="G6" s="65" t="str">
+        <x:v>最大30件まで抽出</x:v>
+      </x:c>
+      <x:c r="H6" s="65"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="E7"/>
+      <x:c r="F7"/>
+      <x:c r="G7"/>
+      <x:c r="H7"/>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="70" t="str">
+        <x:v>改善作業の状況</x:v>
+      </x:c>
+      <x:c r="B8" s="70"/>
+      <x:c r="C8" s="70"/>
+      <x:c r="D8" s="70"/>
+      <x:c r="E8" s="70"/>
+      <x:c r="F8" s="70"/>
+      <x:c r="G8" s="70"/>
+      <x:c r="H8" s="70"/>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="74" t="str">
+        <x:v>項目</x:v>
+      </x:c>
+      <x:c r="B9" s="74" t="str">
+        <x:v>状況</x:v>
+      </x:c>
+      <x:c r="C9"/>
+      <x:c r="D9" s="70" t="str">
         <x:v>今日やること</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" t="str">
-        <x:v>良好記事数</x:v>
-      </x:c>
-      <x:c r="B4" t="n">
-        <x:f>COUNTIF('改善中'!E2:E200,"良好")+COUNTIF('Improvement_Log'!H2:H500,"良好")</x:f>
+      <x:c r="E9" s="70"/>
+      <x:c r="F9" s="70"/>
+      <x:c r="G9" s="70"/>
+      <x:c r="H9" s="70"/>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="77" t="str">
+        <x:v>今日の改善残数</x:v>
+      </x:c>
+      <x:c r="B10" s="77" t="n">
+        <x:f>COUNTIF('今日の改善'!$F$2:$F$6,"未着手")</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C10"/>
+      <x:c r="D10" s="74" t="str">
+        <x:v>優先</x:v>
+      </x:c>
+      <x:c r="E10" s="74" t="str">
+        <x:v>URL</x:v>
+      </x:c>
+      <x:c r="F10" s="74" t="str">
+        <x:v>メインKW</x:v>
+      </x:c>
+      <x:c r="G10" s="74" t="str">
+        <x:v>状態</x:v>
+      </x:c>
+      <x:c r="H10" s="74" t="str">
+        <x:v>操作</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="78" t="str">
+        <x:v>測定中件数</x:v>
+      </x:c>
+      <x:c r="B11" s="78" t="n">
+        <x:f>COUNTIF('改善中'!$E$2:$E$1000,"測定中")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C4" t="str">
-        <x:v>ブログ診断</x:v>
-      </x:c>
-      <x:c r="E4" s="20" t="str">
-        <x:v>優先</x:v>
-      </x:c>
-      <x:c r="F4" s="20" t="str">
-        <x:v>URL</x:v>
-      </x:c>
-      <x:c r="G4" s="20" t="str">
-        <x:v>メインKW</x:v>
-      </x:c>
-      <x:c r="H4" s="20" t="str">
-        <x:v>状態</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str">
-        <x:v>改善中記事数</x:v>
-      </x:c>
-      <x:c r="B5" t="n">
-        <x:f>COUNTA('改善中'!A2:A200)</x:f>
+      <x:c r="C11"/>
+      <x:c r="D11" s="81" t="str">
+        <x:f>IF('今日の改善'!$B2="","",'今日の改善'!$A2)</x:f>
+      </x:c>
+      <x:c r="E11" s="81" t="str">
+        <x:f>IF('今日の改善'!$B2="","",'今日の改善'!$B2)</x:f>
+      </x:c>
+      <x:c r="F11" s="81" t="str">
+        <x:f>IF('今日の改善'!$B2="","",'今日の改善'!$C2)</x:f>
+      </x:c>
+      <x:c r="G11" s="81" t="str">
+        <x:f>IF('今日の改善'!$B2="","",'今日の改善'!$F2)</x:f>
+      </x:c>
+      <x:c r="H11" s="81" t="str">
+        <x:v>改善後、完了</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="A12" s="78" t="str">
+        <x:v>今週の完了件数</x:v>
+      </x:c>
+      <x:c r="B12" s="78" t="n">
+        <x:f>COUNTIFS(Improvement_Log!$E:$E,"&gt;="&amp;TODAY()-WEEKDAY(TODAY(),2)+1,Improvement_Log!$E:$E,"&lt;="&amp;TODAY())</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C5" t="str">
-        <x:v>改善中</x:v>
-      </x:c>
-      <x:c r="E5" t="str">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F5" t="str">
-        <x:f>IFERROR('今日の改善'!B2,"")</x:f>
-      </x:c>
-      <x:c r="G5" t="str">
-        <x:f>IFERROR('今日の改善'!C2,"")</x:f>
-      </x:c>
-      <x:c r="H5" t="str">
-        <x:f>IFERROR('今日の改善'!F2,"")</x:f>
-        <x:v>未着手</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" t="str">
-        <x:v>改善候補数</x:v>
-      </x:c>
-      <x:c r="B6" t="n">
-        <x:f>COUNTA('Improvement_Queue'!A2:A500)</x:f>
+      <x:c r="C12"/>
+      <x:c r="D12" s="82" t="str">
+        <x:f>IF('今日の改善'!$B3="","",'今日の改善'!$A3)</x:f>
+      </x:c>
+      <x:c r="E12" s="82" t="str">
+        <x:f>IF('今日の改善'!$B3="","",'今日の改善'!$B3)</x:f>
+      </x:c>
+      <x:c r="F12" s="82" t="str">
+        <x:f>IF('今日の改善'!$B3="","",'今日の改善'!$C3)</x:f>
+      </x:c>
+      <x:c r="G12" s="82" t="str">
+        <x:f>IF('今日の改善'!$B3="","",'今日の改善'!$F3)</x:f>
+      </x:c>
+      <x:c r="H12" s="82" t="str">
+        <x:v>改善後、完了</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="78" t="str">
+        <x:v>最終データ更新</x:v>
+      </x:c>
+      <x:c r="B13" s="87" t="n">
+        <x:f>IFERROR(MAX(SearchConsole_Data!$A:$A),"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C6" t="str">
-        <x:v>Improvement_Queue</x:v>
-      </x:c>
-      <x:c r="E6" t="str">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F6" t="str">
-        <x:f>IFERROR('今日の改善'!B3,"")</x:f>
-      </x:c>
-      <x:c r="G6" t="str">
-        <x:f>IFERROR('今日の改善'!C3,"")</x:f>
-      </x:c>
-      <x:c r="H6" t="str">
-        <x:f>IFERROR('今日の改善'!F3,"")</x:f>
-        <x:v>未着手</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="E7" t="str">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F7" t="str">
-        <x:f>IFERROR('今日の改善'!B4,"")</x:f>
-      </x:c>
-      <x:c r="G7" t="str">
-        <x:f>IFERROR('今日の改善'!C4,"")</x:f>
-      </x:c>
-      <x:c r="H7" t="str">
-        <x:f>IFERROR('今日の改善'!F4,"")</x:f>
-        <x:v>未着手</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="13" t="str">
-        <x:v>改善作業の状況</x:v>
-      </x:c>
-      <x:c r="B8" s="13" t="str">
-        <x:v>内容</x:v>
-      </x:c>
-      <x:c r="C8" s="13" t="str">
-        <x:v>備考</x:v>
-      </x:c>
-      <x:c r="E8" t="str">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F8" t="str">
-        <x:f>IFERROR('今日の改善'!B5,"")</x:f>
-      </x:c>
-      <x:c r="G8" t="str">
-        <x:f>IFERROR('今日の改善'!C5,"")</x:f>
-      </x:c>
-      <x:c r="H8" t="str">
-        <x:f>IFERROR('今日の改善'!F5,"")</x:f>
-        <x:v>未着手</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" t="str">
-        <x:v>最終取得</x:v>
-      </x:c>
-      <x:c r="B9" t="n">
-        <x:f>IFERROR(MAX('処理ログ'!A2:A200),"未実行")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C9" t="str">
-        <x:v>Search Console</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>今日の改善残数</x:v>
-      </x:c>
-      <x:c r="B10" t="n">
-        <x:f>COUNTA('今日の改善'!A2:A6)</x:f>
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="C10" t="str">
-        <x:v>5件を上限表示</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>測定対象</x:v>
-      </x:c>
-      <x:c r="B11" t="n">
-        <x:f>COUNTA('改善中'!A2:A200)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C11" t="str">
-        <x:v>週1回・最大2か月</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>最終ログ</x:v>
-      </x:c>
-      <x:c r="B12" t="str">
-        <x:f>IFERROR(INDEX('処理ログ'!B2:B200,COUNTA('処理ログ'!B2:B200)),"なし")</x:f>
-      </x:c>
-      <x:c r="C12" t="str"/>
+      <x:c r="D13" s="82" t="str">
+        <x:f>IF('今日の改善'!$B4="","",'今日の改善'!$A4)</x:f>
+      </x:c>
+      <x:c r="E13" s="82" t="str">
+        <x:f>IF('今日の改善'!$B4="","",'今日の改善'!$B4)</x:f>
+      </x:c>
+      <x:c r="F13" s="82" t="str">
+        <x:f>IF('今日の改善'!$B4="","",'今日の改善'!$C4)</x:f>
+      </x:c>
+      <x:c r="G13" s="82" t="str">
+        <x:f>IF('今日の改善'!$B4="","",'今日の改善'!$F4)</x:f>
+      </x:c>
+      <x:c r="H13" s="82" t="str">
+        <x:v>改善後、完了</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="78" t="str">
+        <x:v>最終処理結果</x:v>
+      </x:c>
+      <x:c r="B14" s="78" t="str">
+        <x:f>IFERROR(INDEX('処理ログ'!$F:$F,MATCH(2,1/('処理ログ'!$F:$F&lt;&gt;""))),"")</x:f>
+      </x:c>
+      <x:c r="D14" s="82" t="str">
+        <x:f>IF('今日の改善'!$B5="","",'今日の改善'!$A5)</x:f>
+      </x:c>
+      <x:c r="E14" s="82" t="str">
+        <x:f>IF('今日の改善'!$B5="","",'今日の改善'!$B5)</x:f>
+      </x:c>
+      <x:c r="F14" s="82" t="str">
+        <x:f>IF('今日の改善'!$B5="","",'今日の改善'!$C5)</x:f>
+      </x:c>
+      <x:c r="G14" s="82" t="str">
+        <x:f>IF('今日の改善'!$B5="","",'今日の改善'!$F5)</x:f>
+      </x:c>
+      <x:c r="H14" s="82" t="str">
+        <x:v>改善後、完了</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="D15" s="82" t="str">
+        <x:f>IF('今日の改善'!$B6="","",'今日の改善'!$A6)</x:f>
+      </x:c>
+      <x:c r="E15" s="82" t="str">
+        <x:f>IF('今日の改善'!$B6="","",'今日の改善'!$B6)</x:f>
+      </x:c>
+      <x:c r="F15" s="82" t="str">
+        <x:f>IF('今日の改善'!$B6="","",'今日の改善'!$C6)</x:f>
+      </x:c>
+      <x:c r="G15" s="82" t="str">
+        <x:f>IF('今日の改善'!$B6="","",'今日の改善'!$F6)</x:f>
+      </x:c>
+      <x:c r="H15" s="82" t="str">
+        <x:v>改善後、完了</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="36" customHeight="1">
+      <x:c r="A17" s="86" t="str">
+        <x:v>使い方：まずHomeで状況を確認し、今日の改善を開いて上位5件だけ対応します。完了後は改善中へ移動し、週1回・最大2か月測定します。</x:v>
+      </x:c>
+      <x:c r="B17" s="86"/>
+      <x:c r="C17" s="86"/>
+      <x:c r="D17" s="86"/>
+      <x:c r="E17" s="86"/>
+      <x:c r="F17" s="86"/>
+      <x:c r="G17" s="86"/>
+      <x:c r="H17" s="86"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="E3:H3"/>
+    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A4:B4"/>
+    <x:mergeCell ref="D4:E4"/>
+    <x:mergeCell ref="G4:H4"/>
+    <x:mergeCell ref="A5:B5"/>
+    <x:mergeCell ref="D5:E5"/>
+    <x:mergeCell ref="G5:H5"/>
+    <x:mergeCell ref="A6:B6"/>
+    <x:mergeCell ref="D6:E6"/>
+    <x:mergeCell ref="G6:H6"/>
+    <x:mergeCell ref="A8:H8"/>
+    <x:mergeCell ref="D9:H9"/>
+    <x:mergeCell ref="A17:H17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Product 5.0 Home Phase 1 Fix
</commit_message>
<xml_diff>
--- a/spreadsheet/SIMS-Blog-Manager.xlsx
+++ b/spreadsheet/SIMS-Blog-Manager.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Home" sheetId="1" r:id="R6fc33a1f713a465a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rb8b33ffe38954ab9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善中" sheetId="3" r:id="R3f816bb506274693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ブログ診断" sheetId="4" r:id="R9048189f3efd47c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="処理ログ" sheetId="5" r:id="R7b2b3132cb2547f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設定" sheetId="6" r:id="R6ed0b4f365394cdd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SearchConsole_Data" sheetId="7" r:id="R3885d4aadad84e78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Queue" sheetId="8" r:id="R1d3c6cd1b1c44e66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Log" sheetId="9" r:id="R1189022717c94630"/>
-  </x:sheets>
-</x:workbook>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="Home" sheetId="1" r:id="R1b7d890125d94226"/>
+    <sheet name="今日の改善" sheetId="2" r:id="Rbce89842efa84337"/>
+    <sheet name="改善中" sheetId="3" r:id="Rb110bb684aa7491a"/>
+    <sheet name="ブログ診断" sheetId="4" r:id="R5bc56a9a535c490d"/>
+    <sheet name="処理ログ" sheetId="5" r:id="Rd8d085c92d97490b"/>
+    <sheet name="設定" sheetId="6" r:id="Ra5a08ebd2326493d" state="hidden"/>
+    <sheet name="SearchConsole_Data" sheetId="7" r:id="Rcf45f8f8198c4536" state="hidden"/>
+    <sheet name="Improvement_Queue" sheetId="8" r:id="Re45537a815dc4f6c" state="hidden"/>
+    <sheet name="Improvement_Log" sheetId="9" r:id="R23bcafefd3d94527" state="hidden"/>
+  </sheets>
+</workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -517,8 +517,8 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="3" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="30" hidden="0" customWidth="1"/>
@@ -534,7 +534,9 @@
       <x:c r="A1" s="47" t="str">
         <x:v>SIMS-Blog-Manager Product 5.0 Official</x:v>
       </x:c>
-      <x:c r="B1" s="47"/>
+      <x:c r="B1" s="47" t="str">
+        <x:v>毎日最初に見る画面です。</x:v>
+      </x:c>
       <x:c r="C1" s="47"/>
       <x:c r="D1" s="47"/>
       <x:c r="E1" s="47"/>
@@ -547,9 +549,11 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="50" t="str">
-        <x:v>毎日最初に見る画面：ブログ全体・改善状況・今日やることだけを表示します。</x:v>
-      </x:c>
-      <x:c r="B2" s="50"/>
+        <x:v>バージョン</x:v>
+      </x:c>
+      <x:c r="B2" s="50" t="str">
+        <x:v>5.0.0-official</x:v>
+      </x:c>
       <x:c r="C2" s="50"/>
       <x:c r="D2" s="50"/>
       <x:c r="E2" s="50"/>
@@ -558,16 +562,16 @@
       <x:c r="H2" s="50"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="13"/>
-      <x:c r="B3" s="13"/>
+      <x:c r="A3" s="13" t="str"/>
+      <x:c r="B3" s="13" t="str"/>
       <x:c r="C3" s="13"/>
       <x:c r="E3" s="13"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="55" t="str">
-        <x:v>良好記事数</x:v>
-      </x:c>
-      <x:c r="B4" s="55"/>
+        <x:v>1. ブログ全体の状況</x:v>
+      </x:c>
+      <x:c r="B4" s="55" t="str"/>
       <x:c r="C4"/>
       <x:c r="D4" s="55" t="str">
         <x:v>改善中記事数</x:v>
@@ -580,11 +584,12 @@
       <x:c r="H4" s="55"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="62" t="n">
-        <x:f>COUNTIF('ブログ診断'!$A:$A,"良好")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B5" s="62"/>
+      <x:c r="A5" s="62" t="str">
+        <x:v>総記事数</x:v>
+      </x:c>
+      <x:c r="B5" s="62" t="str">
+        <x:v>0件</x:v>
+      </x:c>
       <x:c r="C5"/>
       <x:c r="D5" s="62" t="n">
         <x:f>COUNTA('改善中'!$B$2:$B$1000)</x:f>
@@ -600,9 +605,11 @@
     </x:row>
     <x:row r="6" ht="22" customHeight="1">
       <x:c r="A6" s="65" t="str">
-        <x:v>当面の改善不要</x:v>
-      </x:c>
-      <x:c r="B6" s="65"/>
+        <x:v>良好記事数</x:v>
+      </x:c>
+      <x:c r="B6" s="65" t="str">
+        <x:v>0件 / 0件（0%）</x:v>
+      </x:c>
       <x:c r="C6"/>
       <x:c r="D6" s="65" t="str">
         <x:v>週1回・最大2か月測定</x:v>
@@ -615,6 +622,12 @@
       <x:c r="H6" s="65"/>
     </x:row>
     <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>改善中記事数</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>0件</x:v>
+      </x:c>
       <x:c r="E7"/>
       <x:c r="F7"/>
       <x:c r="G7"/>
@@ -622,9 +635,11 @@
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="70" t="str">
-        <x:v>改善作業の状況</x:v>
-      </x:c>
-      <x:c r="B8" s="70"/>
+        <x:v>改善候補数</x:v>
+      </x:c>
+      <x:c r="B8" s="70" t="str">
+        <x:v>0件</x:v>
+      </x:c>
       <x:c r="C8" s="70"/>
       <x:c r="D8" s="70"/>
       <x:c r="E8" s="70"/>
@@ -633,12 +648,8 @@
       <x:c r="H8" s="70"/>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="74" t="str">
-        <x:v>項目</x:v>
-      </x:c>
-      <x:c r="B9" s="74" t="str">
-        <x:v>状況</x:v>
-      </x:c>
+      <x:c r="A9" s="74" t="str"/>
+      <x:c r="B9" s="74" t="str"/>
       <x:c r="C9"/>
       <x:c r="D9" s="70" t="str">
         <x:v>今日やること</x:v>
@@ -650,12 +661,9 @@
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="77" t="str">
-        <x:v>今日の改善残数</x:v>
-      </x:c>
-      <x:c r="B10" s="77" t="n">
-        <x:f>COUNTIF('今日の改善'!$F$2:$F$6,"未着手")</x:f>
-        <x:v>5</x:v>
-      </x:c>
+        <x:v>2. 改善作業の状況</x:v>
+      </x:c>
+      <x:c r="B10" s="77" t="str"/>
       <x:c r="C10"/>
       <x:c r="D10" s="74" t="str">
         <x:v>優先</x:v>
@@ -675,11 +683,10 @@
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
       <x:c r="A11" s="78" t="str">
-        <x:v>測定中件数</x:v>
-      </x:c>
-      <x:c r="B11" s="78" t="n">
-        <x:f>COUNTIF('改善中'!$E$2:$E$1000,"測定中")</x:f>
-        <x:v>0</x:v>
+        <x:v>今日の改善表示</x:v>
+      </x:c>
+      <x:c r="B11" s="78" t="str">
+        <x:v>0件</x:v>
       </x:c>
       <x:c r="C11"/>
       <x:c r="D11" s="81" t="str">
@@ -700,11 +707,10 @@
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
       <x:c r="A12" s="78" t="str">
-        <x:v>今週の完了件数</x:v>
-      </x:c>
-      <x:c r="B12" s="78" t="n">
-        <x:f>COUNTIFS(Improvement_Log!$E:$E,"&gt;="&amp;TODAY()-WEEKDAY(TODAY(),2)+1,Improvement_Log!$E:$E,"&lt;="&amp;TODAY())</x:f>
-        <x:v>0</x:v>
+        <x:v>最終取得日</x:v>
+      </x:c>
+      <x:c r="B12" s="78" t="str">
+        <x:v>未取得</x:v>
       </x:c>
       <x:c r="C12"/>
       <x:c r="D12" s="82" t="str">
@@ -725,11 +731,10 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="78" t="str">
-        <x:v>最終データ更新</x:v>
-      </x:c>
-      <x:c r="B13" s="87" t="n">
-        <x:f>IFERROR(MAX(SearchConsole_Data!$A:$A),"")</x:f>
-        <x:v>0</x:v>
+        <x:v>直近処理</x:v>
+      </x:c>
+      <x:c r="B13" s="87" t="str">
+        <x:v>未実行</x:v>
       </x:c>
       <x:c r="D13" s="82" t="str">
         <x:f>IF('今日の改善'!$B4="","",'今日の改善'!$A4)</x:f>
@@ -748,12 +753,8 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
-      <x:c r="A14" s="78" t="str">
-        <x:v>最終処理結果</x:v>
-      </x:c>
-      <x:c r="B14" s="78" t="str">
-        <x:f>IFERROR(INDEX('処理ログ'!$F:$F,MATCH(2,1/('処理ログ'!$F:$F&lt;&gt;""))),"")</x:f>
-      </x:c>
+      <x:c r="A14" s="78" t="str"/>
+      <x:c r="B14" s="78" t="str"/>
       <x:c r="D14" s="82" t="str">
         <x:f>IF('今日の改善'!$B5="","",'今日の改善'!$A5)</x:f>
       </x:c>
@@ -771,6 +772,10 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" t="str">
+        <x:v>3. 今日やること</x:v>
+      </x:c>
+      <x:c r="B15" t="str"/>
       <x:c r="D15" s="82" t="str">
         <x:f>IF('今日の改善'!$B6="","",'今日の改善'!$A6)</x:f>
       </x:c>
@@ -787,17 +792,35 @@
         <x:v>改善後、完了</x:v>
       </x:c>
     </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>次にやること</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>セットアップまたは今日の改善を確認してください。</x:v>
+      </x:c>
+    </x:row>
     <x:row r="17" ht="36" customHeight="1">
       <x:c r="A17" s="86" t="str">
-        <x:v>使い方：まずHomeで状況を確認し、今日の改善を開いて上位5件だけ対応します。完了後は改善中へ移動し、週1回・最大2か月測定します。</x:v>
-      </x:c>
-      <x:c r="B17" s="86"/>
+        <x:v>おすすめ改善</x:v>
+      </x:c>
+      <x:c r="B17" s="86" t="str">
+        <x:v>未作成</x:v>
+      </x:c>
       <x:c r="C17" s="86"/>
       <x:c r="D17" s="86"/>
       <x:c r="E17" s="86"/>
       <x:c r="F17" s="86"/>
       <x:c r="G17" s="86"/>
       <x:c r="H17" s="86"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>推定時間</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>-</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -840,28 +863,28 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="40" t="str">
-        <x:v>優先度</x:v>
+        <x:v>優先</x:v>
       </x:c>
       <x:c r="B1" s="40" t="str">
-        <x:v>URL</x:v>
+        <x:v>時間</x:v>
       </x:c>
       <x:c r="C1" s="40" t="str">
-        <x:v>メインKW</x:v>
+        <x:v>記事タイトル</x:v>
       </x:c>
       <x:c r="D1" s="40" t="str">
-        <x:v>参考クエリ</x:v>
+        <x:v>メインクエリ</x:v>
       </x:c>
       <x:c r="E1" s="40" t="str">
-        <x:v>改善方針</x:v>
+        <x:v>改善内容</x:v>
       </x:c>
       <x:c r="F1" s="40" t="str">
-        <x:v>状態</x:v>
+        <x:v>改善ブリーフ</x:v>
       </x:c>
       <x:c r="G1" s="40" t="str">
-        <x:v>改善完了</x:v>
+        <x:v>完了</x:v>
       </x:c>
       <x:c r="H1" s="40" t="str">
-        <x:v>更新日</x:v>
+        <x:v>メモ</x:v>
       </x:c>
       <x:c r="I1" s="35"/>
       <x:c r="J1" s="35"/>
@@ -4442,9 +4465,9 @@
       <x:c r="A4" t="str">
         <x:v>改善中記事数</x:v>
       </x:c>
-      <x:c r="B4" t="n">
+      <x:c r="B4" t="str">
         <x:f>'Home'!B5</x:f>
-        <x:v>0</x:v>
+        <x:v>0件</x:v>
       </x:c>
       <x:c r="D4" t="str">
         <x:v>良好</x:v>
@@ -4460,9 +4483,9 @@
       <x:c r="A5" t="str">
         <x:v>改善候補数</x:v>
       </x:c>
-      <x:c r="B5" t="n">
+      <x:c r="B5" t="str">
         <x:f>'Home'!B6</x:f>
-        <x:v>0</x:v>
+        <x:v>0件 / 0件（0%）</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>改善中</x:v>

</xml_diff>

<commit_message>
Product 5.0 Clean Menus Home Visual
</commit_message>
<xml_diff>
--- a/spreadsheet/SIMS-Blog-Manager.xlsx
+++ b/spreadsheet/SIMS-Blog-Manager.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Home" sheetId="1" r:id="R921f1f42f20645a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R05716c06eb4e4407"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善中" sheetId="3" r:id="R457f57bf1c394851"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ブログ診断" sheetId="4" r:id="R3e4f16285e3f486f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="処理ログ" sheetId="5" r:id="R8c01573f31544631"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設定" sheetId="6" r:id="Raf138726b67e4907"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SearchConsole_Data" sheetId="7" r:id="R8a04746a589f452c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Queue" sheetId="8" r:id="R81158988c3eb43c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Log" sheetId="9" r:id="R707d769a7cae498b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="データ一覧" sheetId="10" r:id="Rabeee53e3ef14171"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Home" sheetId="1" r:id="R9f15b9ef3b394287"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R98bc516937854b9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善中" sheetId="3" r:id="R9ed568a4ee144019"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ブログ診断" sheetId="4" r:id="R2c9868526fd24349"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="処理ログ" sheetId="5" r:id="R6964c9b565ea4168"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設定" sheetId="6" r:id="R93bb3ad57f124698"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SearchConsole_Data" sheetId="7" r:id="Rd0dba2a086064055"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Queue" sheetId="8" r:id="Rd26e2ecef72b4903"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Log" sheetId="9" r:id="R9767a2ac99834994"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="データ一覧" sheetId="10" r:id="R66345da6b3934092"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="11" r:id="R899a0755af3a437e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28,7 +29,7 @@
     <x:numFmt numFmtId="200" formatCode="0.00%"/>
     <x:numFmt numFmtId="201" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="20">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -89,8 +90,59 @@
       <x:color rgb="FF9A3412"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="22"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFD1D5DB"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF111827"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="20"/>
+      <x:color rgb="FF374151"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF374151"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF374151"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="13"/>
+      <x:color rgb="FF111827"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="12"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -142,6 +194,46 @@
         <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B1324"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111827"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1D4ED8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF59E0B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF9FAFB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFBEB"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -168,7 +260,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="169">
+  <x:cellXfs count="250">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
@@ -557,6 +649,229 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="15" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="18" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="19" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -782,10 +1097,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" style="42" customWidth="1"/>
-    <x:col min="2" max="2" width="72" style="42" customWidth="1"/>
-    <x:col min="3" max="3" width="3" style="42" customWidth="1"/>
-    <x:col min="4" max="4" width="8" style="42" customWidth="1"/>
+    <x:col min="1" max="1" width="18" style="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="44" style="42" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" style="42" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="44" style="42" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="30" style="42" customWidth="1"/>
     <x:col min="6" max="6" width="16" style="42" customWidth="1"/>
     <x:col min="7" max="7" width="12" style="42" customWidth="1"/>
@@ -795,346 +1110,221 @@
     <x:col min="11" max="11" width="18" style="42" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" s="42" customFormat="1" ht="32" customHeight="1">
-      <x:c r="A1" s="88" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SIMS-Blog-Manager Product 5.0 Official</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="1" t="n"/>
-      <x:c r="C1" s="1" t="n"/>
-      <x:c r="D1" s="1" t="n"/>
-      <x:c r="E1" s="1" t="n"/>
-      <x:c r="F1" s="1" t="n"/>
-      <x:c r="G1" s="1" t="n"/>
-      <x:c r="H1" s="1" t="n"/>
+    <x:row r="1" s="42" customFormat="1" ht="42" customHeight="1">
+      <x:c r="A1" s="173" t="str">
+        <x:v>SIMS-Blog-Manager</x:v>
+      </x:c>
+      <x:c r="B1" s="175" t="str">
+        <x:v>Product 5.0 Official</x:v>
+      </x:c>
+      <x:c r="C1" s="175" t="str"/>
+      <x:c r="D1" s="175" t="str"/>
+      <x:c r="E1" s="1"/>
+      <x:c r="F1" s="1"/>
+      <x:c r="G1" s="1"/>
+      <x:c r="H1" s="1"/>
       <x:c r="I1" s="35" t="n"/>
       <x:c r="J1" s="35" t="n"/>
       <x:c r="K1" s="35" t="n"/>
     </x:row>
-    <x:row r="2" s="42" customFormat="1" ht="24" customHeight="1">
-      <x:c r="A2" s="89" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">バージョン</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B2" s="1" t="n"/>
-      <x:c r="C2" s="1" t="n"/>
-      <x:c r="D2" s="1" t="n"/>
-      <x:c r="E2" s="1" t="n"/>
-      <x:c r="F2" s="1" t="n"/>
-      <x:c r="G2" s="1" t="n"/>
-      <x:c r="H2" s="1" t="n"/>
+    <x:row r="2" s="42" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A2" s="180" t="str">
+        <x:v>毎日最初に見る画面</x:v>
+      </x:c>
+      <x:c r="B2" s="180" t="str">
+        <x:v>ブログ全体の状況・改善作業の状況・今日やることだけを表示します。</x:v>
+      </x:c>
+      <x:c r="C2" s="180" t="str"/>
+      <x:c r="D2" s="180" t="str"/>
+      <x:c r="E2" s="1"/>
+      <x:c r="F2" s="1"/>
+      <x:c r="G2" s="1"/>
+      <x:c r="H2" s="1"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="13" t="str"/>
       <x:c r="B3" s="13" t="str"/>
-      <x:c r="C3" s="13" t="n"/>
-      <x:c r="E3" s="17" t="n"/>
-      <x:c r="F3" s="1" t="n"/>
-      <x:c r="G3" s="1" t="n"/>
-      <x:c r="H3" s="1" t="n"/>
-    </x:row>
-    <x:row r="4" s="42" customFormat="1" ht="24" customHeight="1">
-      <x:c r="A4" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1. ブログ全体の状況</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="90" t="n"/>
-      <x:c r="D4" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">改善中記事数</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="90" t="n"/>
-      <x:c r="F4" s="20" t="n"/>
-      <x:c r="G4" s="55" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">改善候補数</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H4" s="90" t="n"/>
+      <x:c r="C3" s="13" t="str"/>
+      <x:c r="D3" t="str"/>
+      <x:c r="E3" s="17"/>
+      <x:c r="F3" s="1"/>
+      <x:c r="G3" s="1"/>
+      <x:c r="H3" s="1"/>
+    </x:row>
+    <x:row r="4" s="42" customFormat="1" ht="34" customHeight="1">
+      <x:c r="A4" s="213" t="str">
+        <x:v>ブログ全体の状況</x:v>
+      </x:c>
+      <x:c r="B4" s="213" t="str"/>
+      <x:c r="C4" s="219" t="str">
+        <x:v>改善作業の状況</x:v>
+      </x:c>
+      <x:c r="D4" s="218" t="str"/>
+      <x:c r="E4" s="90"/>
+      <x:c r="F4" s="20"/>
+      <x:c r="G4" s="55"/>
+      <x:c r="H4" s="90"/>
     </x:row>
     <x:row r="5" s="42" customFormat="1" ht="34" customHeight="1">
-      <x:c r="A5" s="62" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">総記事数</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="75" t="n"/>
-      <x:c r="D5" s="62" t="n">
-        <x:f>COUNTA('改善中'!$B$2:$B$1000)</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E5" s="75" t="n"/>
-      <x:c r="G5" s="62" t="n">
-        <x:f>COUNTIFS(Improvement_Queue!$B:$B,"&lt;&gt;",Improvement_Queue!$I:$I,"&lt;&gt;改善中",Improvement_Queue!$I:$I,"&lt;&gt;測定中",Improvement_Queue!$I:$I,"&lt;&gt;良好",Improvement_Queue!$I:$I,"&lt;&gt;改善不要")</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H5" s="75" t="n"/>
+      <x:c r="A5" s="231" t="str">
+        <x:v>総記事数</x:v>
+      </x:c>
+      <x:c r="B5" s="237" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="C5" s="233" t="str">
+        <x:v>今日の改善表示</x:v>
+      </x:c>
+      <x:c r="D5" s="240" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="E5" s="75"/>
+      <x:c r="G5" s="62"/>
+      <x:c r="H5" s="75"/>
     </x:row>
     <x:row r="6" s="42" customFormat="1" ht="22" customHeight="1">
-      <x:c r="A6" s="91" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">良好記事数</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="1" t="n"/>
-      <x:c r="D6" s="91" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">週1回・最大2か月測定</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" s="1" t="n"/>
-      <x:c r="G6" s="91" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">最大30件まで抽出</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H6" s="1" t="n"/>
+      <x:c r="A6" s="232" t="str">
+        <x:v>良好記事数</x:v>
+      </x:c>
+      <x:c r="B6" s="238" t="str">
+        <x:v>0件 / 0件（0%）</x:v>
+      </x:c>
+      <x:c r="C6" s="233" t="str">
+        <x:v>改善中記事数</x:v>
+      </x:c>
+      <x:c r="D6" s="241" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="E6" s="1"/>
+      <x:c r="G6" s="91"/>
+      <x:c r="H6" s="1"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">改善中記事数</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0件</x:t>
-        </x:is>
+      <x:c r="A7" s="233" t="str">
+        <x:v>改善候補数</x:v>
+      </x:c>
+      <x:c r="B7" s="238" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="C7" s="233" t="str">
+        <x:v>最終取得日</x:v>
+      </x:c>
+      <x:c r="D7" s="238" t="str">
+        <x:v>未取得</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="42" customFormat="1" ht="24" customHeight="1">
-      <x:c r="A8" s="92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">改善候補数</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B8" s="1" t="n"/>
-      <x:c r="C8" s="1" t="n"/>
-      <x:c r="D8" s="1" t="n"/>
-      <x:c r="E8" s="1" t="n"/>
-      <x:c r="F8" s="1" t="n"/>
-      <x:c r="G8" s="1" t="n"/>
-      <x:c r="H8" s="1" t="n"/>
+      <x:c r="A8" s="234" t="str"/>
+      <x:c r="B8" s="239" t="str"/>
+      <x:c r="C8" s="233" t="str">
+        <x:v>直近処理</x:v>
+      </x:c>
+      <x:c r="D8" s="238" t="str">
+        <x:v>未実行</x:v>
+      </x:c>
+      <x:c r="E8" s="1"/>
+      <x:c r="F8" s="1"/>
+      <x:c r="G8" s="1"/>
+      <x:c r="H8" s="1"/>
     </x:row>
     <x:row r="9" s="42" customFormat="1" ht="24" customHeight="1">
       <x:c r="A9" s="74" t="str"/>
       <x:c r="B9" s="74" t="str"/>
-      <x:c r="D9" s="92" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">今日やること</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E9" s="1" t="n"/>
-      <x:c r="F9" s="1" t="n"/>
-      <x:c r="G9" s="1" t="n"/>
-      <x:c r="H9" s="1" t="n"/>
-    </x:row>
-    <x:row r="10" s="42" customFormat="1" ht="24" customHeight="1">
-      <x:c r="A10" s="77" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2. 改善作業の状況</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B10" s="77" t="str"/>
-      <x:c r="D10" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">優先</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">URL</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F10" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">メインKW</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G10" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">状態</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H10" s="74" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">操作</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="C9" t="str"/>
+      <x:c r="D9" s="92" t="str"/>
+      <x:c r="E9" s="1"/>
+      <x:c r="F9" s="1"/>
+      <x:c r="G9" s="1"/>
+      <x:c r="H9" s="1"/>
+    </x:row>
+    <x:row r="10" s="42" customFormat="1" ht="34" customHeight="1">
+      <x:c r="A10" s="226" t="str">
+        <x:v>今日やること</x:v>
+      </x:c>
+      <x:c r="B10" s="226" t="str"/>
+      <x:c r="C10" s="225" t="str"/>
+      <x:c r="D10" s="225" t="str"/>
+      <x:c r="E10" s="74"/>
+      <x:c r="F10" s="74"/>
+      <x:c r="G10" s="74"/>
+      <x:c r="H10" s="74"/>
     </x:row>
     <x:row r="11" s="42" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A11" s="78" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">今日の改善表示</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" s="78" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0件</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D11" s="81" t="str">
-        <x:f>IF('今日の改善'!$B2="","",'今日の改善'!$A2)</x:f>
-      </x:c>
-      <x:c r="E11" s="81" t="str">
-        <x:f>IF('今日の改善'!$B2="","",'今日の改善'!$B2)</x:f>
-      </x:c>
-      <x:c r="F11" s="81" t="str">
-        <x:f>IF('今日の改善'!$B2="","",'今日の改善'!$C2)</x:f>
-      </x:c>
-      <x:c r="G11" s="81" t="str">
-        <x:f>IF('今日の改善'!$B2="","",'今日の改善'!$F2)</x:f>
-      </x:c>
-      <x:c r="H11" s="81" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">改善後、完了</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A11" s="236" t="str">
+        <x:v>次にやること</x:v>
+      </x:c>
+      <x:c r="B11" s="242" t="str">
+        <x:v>セットアップまたは今日の改善を確認してください。</x:v>
+      </x:c>
+      <x:c r="C11" s="243" t="str"/>
+      <x:c r="D11" s="244" t="str"/>
+      <x:c r="E11" s="81"/>
+      <x:c r="F11" s="81"/>
+      <x:c r="G11" s="81"/>
+      <x:c r="H11" s="81"/>
     </x:row>
     <x:row r="12" s="42" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A12" s="78" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">最終取得日</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" s="78" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">未取得</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D12" s="82" t="str">
-        <x:f>IF('今日の改善'!$B3="","",'今日の改善'!$A3)</x:f>
-      </x:c>
-      <x:c r="E12" s="82" t="str">
-        <x:f>IF('今日の改善'!$B3="","",'今日の改善'!$B3)</x:f>
-      </x:c>
-      <x:c r="F12" s="82" t="str">
-        <x:f>IF('今日の改善'!$B3="","",'今日の改善'!$C3)</x:f>
-      </x:c>
-      <x:c r="G12" s="82" t="str">
-        <x:f>IF('今日の改善'!$B3="","",'今日の改善'!$F3)</x:f>
-      </x:c>
-      <x:c r="H12" s="82" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">改善後、完了</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A12" s="236" t="str">
+        <x:v>おすすめ改善</x:v>
+      </x:c>
+      <x:c r="B12" s="242" t="str">
+        <x:v>未作成</x:v>
+      </x:c>
+      <x:c r="C12" s="243" t="str"/>
+      <x:c r="D12" s="242" t="str"/>
+      <x:c r="E12" s="82"/>
+      <x:c r="F12" s="82"/>
+      <x:c r="G12" s="82"/>
+      <x:c r="H12" s="82"/>
     </x:row>
     <x:row r="13" s="42" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A13" s="78" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">直近処理</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" s="93" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">未実行</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D13" s="82" t="str">
-        <x:f>IF('今日の改善'!$B4="","",'今日の改善'!$A4)</x:f>
-      </x:c>
-      <x:c r="E13" s="82" t="str">
-        <x:f>IF('今日の改善'!$B4="","",'今日の改善'!$B4)</x:f>
-      </x:c>
-      <x:c r="F13" s="82" t="str">
-        <x:f>IF('今日の改善'!$B4="","",'今日の改善'!$C4)</x:f>
-      </x:c>
-      <x:c r="G13" s="82" t="str">
-        <x:f>IF('今日の改善'!$B4="","",'今日の改善'!$F4)</x:f>
-      </x:c>
-      <x:c r="H13" s="82" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">改善後、完了</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A13" s="236" t="str">
+        <x:v>推定時間</x:v>
+      </x:c>
+      <x:c r="B13" s="245" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="C13" s="244" t="str"/>
+      <x:c r="D13" s="242" t="str"/>
+      <x:c r="E13" s="82"/>
+      <x:c r="F13" s="82"/>
+      <x:c r="G13" s="82"/>
+      <x:c r="H13" s="82"/>
     </x:row>
     <x:row r="14" s="42" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A14" s="78" t="str"/>
-      <x:c r="B14" s="78" t="str"/>
-      <x:c r="D14" s="82" t="str">
-        <x:f>IF('今日の改善'!$B5="","",'今日の改善'!$A5)</x:f>
-      </x:c>
-      <x:c r="E14" s="82" t="str">
-        <x:f>IF('今日の改善'!$B5="","",'今日の改善'!$B5)</x:f>
-      </x:c>
-      <x:c r="F14" s="82" t="str">
-        <x:f>IF('今日の改善'!$B5="","",'今日の改善'!$C5)</x:f>
-      </x:c>
-      <x:c r="G14" s="82" t="str">
-        <x:f>IF('今日の改善'!$B5="","",'今日の改善'!$F5)</x:f>
-      </x:c>
-      <x:c r="H14" s="82" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">改善後、完了</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A14" s="78"/>
+      <x:c r="B14" s="78"/>
+      <x:c r="D14" s="82"/>
+      <x:c r="E14" s="82"/>
+      <x:c r="F14" s="82"/>
+      <x:c r="G14" s="82"/>
+      <x:c r="H14" s="82"/>
     </x:row>
     <x:row r="15" s="42" customFormat="1" ht="30" customHeight="1">
-      <x:c r="A15" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">3. 今日やること</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D15" s="82" t="str">
-        <x:f>IF('今日の改善'!$B6="","",'今日の改善'!$A6)</x:f>
-      </x:c>
-      <x:c r="E15" s="82" t="str">
-        <x:f>IF('今日の改善'!$B6="","",'今日の改善'!$B6)</x:f>
-      </x:c>
-      <x:c r="F15" s="82" t="str">
-        <x:f>IF('今日の改善'!$B6="","",'今日の改善'!$C6)</x:f>
-      </x:c>
-      <x:c r="G15" s="82" t="str">
-        <x:f>IF('今日の改善'!$B6="","",'今日の改善'!$F6)</x:f>
-      </x:c>
-      <x:c r="H15" s="82" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">改善後、完了</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A15"/>
+      <x:c r="D15" s="82"/>
+      <x:c r="E15" s="82"/>
+      <x:c r="F15" s="82"/>
+      <x:c r="G15" s="82"/>
+      <x:c r="H15" s="82"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">次にやること</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">セットアップまたは今日の改善を確認してください。</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A16"/>
+      <x:c r="B16"/>
     </x:row>
     <x:row r="17" s="42" customFormat="1" ht="36" customHeight="1">
-      <x:c r="A17" s="94" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">おすすめ改善</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B17" s="1" t="n"/>
-      <x:c r="C17" s="1" t="n"/>
-      <x:c r="D17" s="1" t="n"/>
-      <x:c r="E17" s="1" t="n"/>
-      <x:c r="F17" s="1" t="n"/>
-      <x:c r="G17" s="1" t="n"/>
-      <x:c r="H17" s="1" t="n"/>
+      <x:c r="A17" s="94"/>
+      <x:c r="B17" s="1"/>
+      <x:c r="C17" s="1"/>
+      <x:c r="D17" s="1"/>
+      <x:c r="E17" s="1"/>
+      <x:c r="F17" s="1"/>
+      <x:c r="G17" s="1"/>
+      <x:c r="H17" s="1"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">推定時間</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">-</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="A18"/>
+      <x:c r="B18"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1153,6 +1343,10 @@
     <x:mergeCell ref="A6:B6"/>
     <x:mergeCell ref="D9:H9"/>
     <x:mergeCell ref="A17:H17"/>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A2:D2"/>
+    <x:mergeCell ref="C4:D4"/>
+    <x:mergeCell ref="A10:D10"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1200,6 +1394,89 @@
       </x:c>
       <x:c r="I1" s="168" t="str">
         <x:v>平均順位</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="36" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="36" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="36" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="52" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="249" t="str">
+        <x:v>BriefId</x:v>
+      </x:c>
+      <x:c r="B1" s="249" t="str">
+        <x:v>URL</x:v>
+      </x:c>
+      <x:c r="C1" s="249" t="str">
+        <x:v>記事タイトル</x:v>
+      </x:c>
+      <x:c r="D1" s="249" t="str">
+        <x:v>メインクエリ</x:v>
+      </x:c>
+      <x:c r="E1" s="249" t="str">
+        <x:v>サブクエリ</x:v>
+      </x:c>
+      <x:c r="F1" s="249" t="str">
+        <x:v>FAQ候補</x:v>
+      </x:c>
+      <x:c r="G1" s="249" t="str">
+        <x:v>別記事候補</x:v>
+      </x:c>
+      <x:c r="H1" s="249" t="str">
+        <x:v>除外クエリ</x:v>
+      </x:c>
+      <x:c r="I1" s="249" t="str">
+        <x:v>クエリ分析</x:v>
+      </x:c>
+      <x:c r="J1" s="249" t="str">
+        <x:v>カニバリ診断</x:v>
+      </x:c>
+      <x:c r="K1" s="249" t="str">
+        <x:v>診断</x:v>
+      </x:c>
+      <x:c r="L1" s="249" t="str">
+        <x:v>推奨改善</x:v>
+      </x:c>
+      <x:c r="M1" s="249" t="str">
+        <x:v>理由</x:v>
+      </x:c>
+      <x:c r="N1" s="249" t="str">
+        <x:v>推定時間</x:v>
+      </x:c>
+      <x:c r="O1" s="249" t="str">
+        <x:v>Score</x:v>
+      </x:c>
+      <x:c r="P1" s="249" t="str">
+        <x:v>CTR</x:v>
+      </x:c>
+      <x:c r="Q1" s="249" t="str">
+        <x:v>Position</x:v>
+      </x:c>
+      <x:c r="R1" s="249" t="str">
+        <x:v>Clicks</x:v>
+      </x:c>
+      <x:c r="S1" s="249" t="str">
+        <x:v>Impressions</x:v>
+      </x:c>
+      <x:c r="T1" s="249" t="str">
+        <x:v>改善依頼文</x:v>
+      </x:c>
+      <x:c r="U1" s="249" t="str">
+        <x:v>作成日時</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4828,9 +5105,8 @@
           <x:t xml:space="preserve">良好記事数</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="20" t="n">
+      <x:c r="B3" s="20" t="str">
         <x:f>'Home'!B4</x:f>
-        <x:v>0</x:v>
       </x:c>
       <x:c r="D3" s="13" t="inlineStr">
         <x:is>
@@ -4854,9 +5130,9 @@
           <x:t xml:space="preserve">改善中記事数</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" t="n">
+      <x:c r="B4" t="str">
         <x:f>'Home'!B5</x:f>
-        <x:v>0</x:v>
+        <x:v>0件</x:v>
       </x:c>
       <x:c r="D4" t="inlineStr">
         <x:is>
@@ -4880,9 +5156,9 @@
           <x:t xml:space="preserve">改善候補数</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" t="n">
+      <x:c r="B5" t="str">
         <x:f>'Home'!B6</x:f>
-        <x:v>0</x:v>
+        <x:v>0件 / 0件（0%）</x:v>
       </x:c>
       <x:c r="D5" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
Product 5.0 Brief InProgress Phase 2
</commit_message>
<xml_diff>
--- a/spreadsheet/SIMS-Blog-Manager.xlsx
+++ b/spreadsheet/SIMS-Blog-Manager.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Home" sheetId="1" r:id="R9f15b9ef3b394287"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R98bc516937854b9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善中" sheetId="3" r:id="R9ed568a4ee144019"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ブログ診断" sheetId="4" r:id="R2c9868526fd24349"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="処理ログ" sheetId="5" r:id="R6964c9b565ea4168"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設定" sheetId="6" r:id="R93bb3ad57f124698"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SearchConsole_Data" sheetId="7" r:id="Rd0dba2a086064055"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Queue" sheetId="8" r:id="Rd26e2ecef72b4903"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Log" sheetId="9" r:id="R9767a2ac99834994"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="データ一覧" sheetId="10" r:id="R66345da6b3934092"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="11" r:id="R899a0755af3a437e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Home" sheetId="1" r:id="R9b29ab4330254c89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R8424ea6a7e0c4206"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善中" sheetId="3" r:id="Raaa2ffa5ba924334"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ブログ診断" sheetId="4" r:id="R798692b5606c4ac8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="処理ログ" sheetId="5" r:id="Rccfedaedd83a48dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設定" sheetId="6" r:id="R73f2cf0ef9884f47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SearchConsole_Data" sheetId="7" r:id="R24a5eb93c3034b32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Queue" sheetId="8" r:id="R53e3060329e14f16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improvement_Log" sheetId="9" r:id="R75ea0d6507594ab4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="データ一覧" sheetId="10" r:id="Rc991757bf6884991"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="11" r:id="R4add31c164df49bf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -142,7 +142,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="19">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -234,6 +234,16 @@
         <x:fgColor rgb="FFFFFBEB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E79"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B8043"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="5">
     <x:border/>
@@ -260,7 +270,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="250">
+  <x:cellXfs count="262">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
@@ -872,6 +882,38 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1405,79 +1447,272 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="40" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="36" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="36" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="36" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="52" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="10" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="32" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="8" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="30" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="34" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="28" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="8" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="10" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="10" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="10" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="34" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="14" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="249" t="str">
-        <x:v>BriefId</x:v>
-      </x:c>
-      <x:c r="B1" s="249" t="str">
+      <x:c r="A1" s="255" t="str">
+        <x:v>優先度</x:v>
+      </x:c>
+      <x:c r="B1" s="255" t="str">
+        <x:v>記事タイトル</x:v>
+      </x:c>
+      <x:c r="C1" s="255" t="str">
+        <x:v>メインキーワード</x:v>
+      </x:c>
+      <x:c r="D1" s="255" t="str">
+        <x:v>改善内容</x:v>
+      </x:c>
+      <x:c r="E1" s="255" t="str">
+        <x:v>予想時間</x:v>
+      </x:c>
+      <x:c r="F1" s="255" t="str">
+        <x:v>期待効果</x:v>
+      </x:c>
+      <x:c r="G1" s="255" t="str">
+        <x:v>改善依頼（詳細）</x:v>
+      </x:c>
+      <x:c r="H1" s="255" t="str">
         <x:v>URL</x:v>
       </x:c>
-      <x:c r="C1" s="249" t="str">
-        <x:v>記事タイトル</x:v>
-      </x:c>
-      <x:c r="D1" s="249" t="str">
-        <x:v>メインクエリ</x:v>
-      </x:c>
-      <x:c r="E1" s="249" t="str">
+      <x:c r="I1" s="255" t="str">
         <x:v>サブクエリ</x:v>
       </x:c>
-      <x:c r="F1" s="249" t="str">
+      <x:c r="J1" s="255" t="str">
         <x:v>FAQ候補</x:v>
       </x:c>
-      <x:c r="G1" s="249" t="str">
+      <x:c r="K1" s="255" t="str">
         <x:v>別記事候補</x:v>
       </x:c>
-      <x:c r="H1" s="249" t="str">
+      <x:c r="L1" s="255" t="str">
         <x:v>除外クエリ</x:v>
       </x:c>
-      <x:c r="I1" s="249" t="str">
+      <x:c r="M1" s="255" t="str">
         <x:v>クエリ分析</x:v>
       </x:c>
-      <x:c r="J1" s="249" t="str">
-        <x:v>カニバリ診断</x:v>
-      </x:c>
-      <x:c r="K1" s="249" t="str">
-        <x:v>診断</x:v>
-      </x:c>
-      <x:c r="L1" s="249" t="str">
-        <x:v>推奨改善</x:v>
-      </x:c>
-      <x:c r="M1" s="249" t="str">
-        <x:v>理由</x:v>
-      </x:c>
-      <x:c r="N1" s="249" t="str">
-        <x:v>推定時間</x:v>
-      </x:c>
-      <x:c r="O1" s="249" t="str">
+      <x:c r="N1" s="255" t="str">
+        <x:v>改善理由</x:v>
+      </x:c>
+      <x:c r="O1" s="255" t="str">
+        <x:v>具体的な修正方法</x:v>
+      </x:c>
+      <x:c r="P1" s="255" t="str">
+        <x:v>修正例</x:v>
+      </x:c>
+      <x:c r="Q1" s="255" t="str">
         <x:v>Score</x:v>
       </x:c>
-      <x:c r="P1" s="249" t="str">
+      <x:c r="R1" s="255" t="str">
         <x:v>CTR</x:v>
       </x:c>
-      <x:c r="Q1" s="249" t="str">
-        <x:v>Position</x:v>
-      </x:c>
-      <x:c r="R1" s="249" t="str">
-        <x:v>Clicks</x:v>
-      </x:c>
-      <x:c r="S1" s="249" t="str">
-        <x:v>Impressions</x:v>
-      </x:c>
-      <x:c r="T1" s="249" t="str">
-        <x:v>改善依頼文</x:v>
-      </x:c>
-      <x:c r="U1" s="249" t="str">
+      <x:c r="S1" s="255" t="str">
+        <x:v>平均順位</x:v>
+      </x:c>
+      <x:c r="T1" s="255" t="str">
+        <x:v>クリック数</x:v>
+      </x:c>
+      <x:c r="U1" s="255" t="str">
+        <x:v>表示回数</x:v>
+      </x:c>
+      <x:c r="V1" s="258" t="str">
+        <x:v>Claude改善依頼文</x:v>
+      </x:c>
+      <x:c r="W1" s="258" t="str">
         <x:v>作成日時</x:v>
       </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="109"/>
+      <x:c r="B2" s="109"/>
+      <x:c r="C2" s="109"/>
+      <x:c r="D2" s="109"/>
+      <x:c r="E2" s="109"/>
+      <x:c r="F2" s="109"/>
+      <x:c r="G2" s="109"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="109"/>
+      <x:c r="B3" s="109"/>
+      <x:c r="C3" s="109"/>
+      <x:c r="D3" s="109"/>
+      <x:c r="E3" s="109"/>
+      <x:c r="F3" s="109"/>
+      <x:c r="G3" s="109"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="109"/>
+      <x:c r="B4" s="109"/>
+      <x:c r="C4" s="109"/>
+      <x:c r="D4" s="109"/>
+      <x:c r="E4" s="109"/>
+      <x:c r="F4" s="109"/>
+      <x:c r="G4" s="109"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="109"/>
+      <x:c r="B5" s="109"/>
+      <x:c r="C5" s="109"/>
+      <x:c r="D5" s="109"/>
+      <x:c r="E5" s="109"/>
+      <x:c r="F5" s="109"/>
+      <x:c r="G5" s="109"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="109"/>
+      <x:c r="B6" s="109"/>
+      <x:c r="C6" s="109"/>
+      <x:c r="D6" s="109"/>
+      <x:c r="E6" s="109"/>
+      <x:c r="F6" s="109"/>
+      <x:c r="G6" s="109"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="109"/>
+      <x:c r="B7" s="109"/>
+      <x:c r="C7" s="109"/>
+      <x:c r="D7" s="109"/>
+      <x:c r="E7" s="109"/>
+      <x:c r="F7" s="109"/>
+      <x:c r="G7" s="109"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="109"/>
+      <x:c r="B8" s="109"/>
+      <x:c r="C8" s="109"/>
+      <x:c r="D8" s="109"/>
+      <x:c r="E8" s="109"/>
+      <x:c r="F8" s="109"/>
+      <x:c r="G8" s="109"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="109"/>
+      <x:c r="B9" s="109"/>
+      <x:c r="C9" s="109"/>
+      <x:c r="D9" s="109"/>
+      <x:c r="E9" s="109"/>
+      <x:c r="F9" s="109"/>
+      <x:c r="G9" s="109"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="109"/>
+      <x:c r="B10" s="109"/>
+      <x:c r="C10" s="109"/>
+      <x:c r="D10" s="109"/>
+      <x:c r="E10" s="109"/>
+      <x:c r="F10" s="109"/>
+      <x:c r="G10" s="109"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="109"/>
+      <x:c r="B11" s="109"/>
+      <x:c r="C11" s="109"/>
+      <x:c r="D11" s="109"/>
+      <x:c r="E11" s="109"/>
+      <x:c r="F11" s="109"/>
+      <x:c r="G11" s="109"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="109"/>
+      <x:c r="B12" s="109"/>
+      <x:c r="C12" s="109"/>
+      <x:c r="D12" s="109"/>
+      <x:c r="E12" s="109"/>
+      <x:c r="F12" s="109"/>
+      <x:c r="G12" s="109"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="109"/>
+      <x:c r="B13" s="109"/>
+      <x:c r="C13" s="109"/>
+      <x:c r="D13" s="109"/>
+      <x:c r="E13" s="109"/>
+      <x:c r="F13" s="109"/>
+      <x:c r="G13" s="109"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="109"/>
+      <x:c r="B14" s="109"/>
+      <x:c r="C14" s="109"/>
+      <x:c r="D14" s="109"/>
+      <x:c r="E14" s="109"/>
+      <x:c r="F14" s="109"/>
+      <x:c r="G14" s="109"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="109"/>
+      <x:c r="B15" s="109"/>
+      <x:c r="C15" s="109"/>
+      <x:c r="D15" s="109"/>
+      <x:c r="E15" s="109"/>
+      <x:c r="F15" s="109"/>
+      <x:c r="G15" s="109"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="109"/>
+      <x:c r="B16" s="109"/>
+      <x:c r="C16" s="109"/>
+      <x:c r="D16" s="109"/>
+      <x:c r="E16" s="109"/>
+      <x:c r="F16" s="109"/>
+      <x:c r="G16" s="109"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="109"/>
+      <x:c r="B17" s="109"/>
+      <x:c r="C17" s="109"/>
+      <x:c r="D17" s="109"/>
+      <x:c r="E17" s="109"/>
+      <x:c r="F17" s="109"/>
+      <x:c r="G17" s="109"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="109"/>
+      <x:c r="B18" s="109"/>
+      <x:c r="C18" s="109"/>
+      <x:c r="D18" s="109"/>
+      <x:c r="E18" s="109"/>
+      <x:c r="F18" s="109"/>
+      <x:c r="G18" s="109"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="109"/>
+      <x:c r="B19" s="109"/>
+      <x:c r="C19" s="109"/>
+      <x:c r="D19" s="109"/>
+      <x:c r="E19" s="109"/>
+      <x:c r="F19" s="109"/>
+      <x:c r="G19" s="109"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="109"/>
+      <x:c r="B20" s="109"/>
+      <x:c r="C20" s="109"/>
+      <x:c r="D20" s="109"/>
+      <x:c r="E20" s="109"/>
+      <x:c r="F20" s="109"/>
+      <x:c r="G20" s="109"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1624,52 +1859,36 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="42" customFormat="1" ht="28" customHeight="1">
-      <x:c r="A1" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">記事ID</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">URL</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C1" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">メインKW</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D1" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">改善実施日</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E1" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">状態</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F1" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">次回測定日</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G1" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">測定終了日</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H1" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">経過週</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I1" s="40" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">メモ</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J1" s="35" t="n"/>
+      <x:c r="A1" s="259" t="str">
+        <x:v>改善日</x:v>
+      </x:c>
+      <x:c r="B1" s="259" t="str">
+        <x:v>記事タイトル</x:v>
+      </x:c>
+      <x:c r="C1" s="259" t="str">
+        <x:v>経過日数</x:v>
+      </x:c>
+      <x:c r="D1" s="259" t="str">
+        <x:v>状態</x:v>
+      </x:c>
+      <x:c r="E1" s="259" t="str">
+        <x:v>SIMS評価</x:v>
+      </x:c>
+      <x:c r="F1" s="259" t="str">
+        <x:v>次のアクション</x:v>
+      </x:c>
+      <x:c r="G1" s="259" t="str">
+        <x:v>詳細</x:v>
+      </x:c>
+      <x:c r="H1" s="259" t="str">
+        <x:v>URL</x:v>
+      </x:c>
+      <x:c r="I1" s="259" t="str">
+        <x:v>修正内容</x:v>
+      </x:c>
+      <x:c r="J1" s="261" t="str">
+        <x:v>改善内容</x:v>
+      </x:c>
       <x:c r="K1" s="35" t="n"/>
     </x:row>
     <x:row r="2">
@@ -5105,8 +5324,9 @@
           <x:t xml:space="preserve">良好記事数</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="20" t="str">
+      <x:c r="B3" s="20" t="n">
         <x:f>'Home'!B4</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D3" s="13" t="inlineStr">
         <x:is>

</xml_diff>